<commit_message>
Update AI marks calibrated with actual song listening and human evaluator observations
</commit_message>
<xml_diff>
--- a/Judges_Scoring_Sheet.xlsx
+++ b/Judges_Scoring_Sheet.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,7 +42,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -53,12 +52,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="9.5"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -106,8 +100,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
-        <bgColor rgb="00F8FAFC"/>
+        <fgColor rgb="00FAFAFA"/>
+        <bgColor rgb="00FAFAFA"/>
       </patternFill>
     </fill>
     <fill>
@@ -153,16 +147,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00CCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00CCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00CCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
@@ -190,37 +184,37 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -615,11 +609,10 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Framework: AI Benchmark (40 Marks) + Human Judges Live Defense (60 Marks: Creativity 20M, Music Composition 20M, Emotional Impact 10M, Presentation 10M)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="6" customHeight="1"/>
+          <t>Framework: AI Benchmark (40 Marks, Audio-Calibrated) + Human Judges Live Defense (60 Marks: Creativity 20M, Music Composition 20M, Emotional Impact 10M, Presentation 10M)</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -652,8 +645,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1"/>
-    <row r="6" ht="18" customHeight="1">
+    <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>#</t>
@@ -677,7 +669,7 @@
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>PART B: Human Judges Live Defense (60M)</t>
+          <t>PART B: Human Judges Live Scoring (60M)</t>
         </is>
       </c>
       <c r="G6" s="6" t="n"/>
@@ -702,7 +694,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="26" customHeight="1">
+    <row r="7">
       <c r="A7" s="4" t="n"/>
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="4" t="n"/>
@@ -760,11 +752,11 @@
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>33.5</v>
+        <v>35</v>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>83.8%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr"/>
@@ -796,11 +788,11 @@
         </is>
       </c>
       <c r="D9" s="11" t="n">
-        <v>29.5</v>
+        <v>30.5</v>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>73.8%</t>
+          <t>76.2%</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr"/>
@@ -832,11 +824,11 @@
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>31</v>
+        <v>32.5</v>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>77.5%</t>
+          <t>81.2%</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr"/>
@@ -904,11 +896,11 @@
         </is>
       </c>
       <c r="D12" s="11" t="n">
-        <v>31</v>
+        <v>31.5</v>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>77.5%</t>
+          <t>78.8%</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr"/>
@@ -940,11 +932,11 @@
         </is>
       </c>
       <c r="D13" s="11" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>72.5%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr"/>
@@ -976,11 +968,11 @@
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>65.0%</t>
+          <t>62.5%</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr"/>
@@ -1012,11 +1004,11 @@
         </is>
       </c>
       <c r="D15" s="11" t="n">
-        <v>31.5</v>
+        <v>32.5</v>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>78.8%</t>
+          <t>81.2%</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr"/>
@@ -1084,11 +1076,11 @@
         </is>
       </c>
       <c r="D17" s="11" t="n">
-        <v>24.5</v>
+        <v>23.5</v>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>61.3%</t>
+          <t>58.8%</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr"/>
@@ -1120,11 +1112,11 @@
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>29.5</v>
+        <v>26.5</v>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>73.8%</t>
+          <t>66.2%</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr"/>
@@ -1156,11 +1148,11 @@
         </is>
       </c>
       <c r="D19" s="11" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>72.5%</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr"/>
@@ -1192,11 +1184,11 @@
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>27.5</v>
+        <v>25.5</v>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>68.8%</t>
+          <t>63.7%</t>
         </is>
       </c>
       <c r="F20" s="13" t="inlineStr"/>
@@ -1228,11 +1220,11 @@
         </is>
       </c>
       <c r="D21" s="11" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>62.5%</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr"/>
@@ -1264,11 +1256,11 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>26</v>
+        <v>24.5</v>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>65.0%</t>
+          <t>61.3%</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr"/>
@@ -1300,11 +1292,11 @@
         </is>
       </c>
       <c r="D23" s="11" t="n">
-        <v>32</v>
+        <v>25.5</v>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>63.7%</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr"/>
@@ -1336,11 +1328,11 @@
         </is>
       </c>
       <c r="D24" s="11" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>82.5%</t>
         </is>
       </c>
       <c r="F24" s="13" t="inlineStr"/>
@@ -1372,11 +1364,11 @@
         </is>
       </c>
       <c r="D25" s="11" t="n">
-        <v>31.5</v>
+        <v>29.5</v>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>78.8%</t>
+          <t>73.8%</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr"/>
@@ -1444,11 +1436,11 @@
         </is>
       </c>
       <c r="D27" s="11" t="n">
-        <v>32.5</v>
+        <v>31</v>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>81.2%</t>
+          <t>77.5%</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr"/>
@@ -1480,11 +1472,11 @@
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>29.5</v>
+        <v>27</v>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>73.8%</t>
+          <t>67.5%</t>
         </is>
       </c>
       <c r="F28" s="13" t="inlineStr"/>
@@ -1516,11 +1508,11 @@
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>47.5%</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr"/>
@@ -1588,11 +1580,11 @@
         </is>
       </c>
       <c r="D31" s="11" t="n">
-        <v>31</v>
+        <v>29.5</v>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>77.5%</t>
+          <t>73.8%</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr"/>
@@ -1624,11 +1616,11 @@
         </is>
       </c>
       <c r="D32" s="11" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>92.5%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr"/>
@@ -1660,11 +1652,11 @@
         </is>
       </c>
       <c r="D33" s="11" t="n">
-        <v>19.5</v>
+        <v>16</v>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>48.8%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F33" s="13" t="inlineStr"/>
@@ -1696,11 +1688,11 @@
         </is>
       </c>
       <c r="D34" s="11" t="n">
-        <v>26</v>
+        <v>21.5</v>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>65.0%</t>
+          <t>53.8%</t>
         </is>
       </c>
       <c r="F34" s="13" t="inlineStr"/>
@@ -1732,11 +1724,11 @@
         </is>
       </c>
       <c r="D35" s="11" t="n">
-        <v>34</v>
+        <v>25.5</v>
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>85.0%</t>
+          <t>63.7%</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr"/>
@@ -1768,11 +1760,11 @@
         </is>
       </c>
       <c r="D36" s="11" t="n">
-        <v>34.5</v>
+        <v>26</v>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>86.2%</t>
+          <t>65.0%</t>
         </is>
       </c>
       <c r="F36" s="13" t="inlineStr"/>
@@ -1804,11 +1796,11 @@
         </is>
       </c>
       <c r="D37" s="11" t="n">
-        <v>36</v>
+        <v>34.5</v>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>90.0%</t>
+          <t>86.2%</t>
         </is>
       </c>
       <c r="F37" s="13" t="inlineStr"/>
@@ -1840,11 +1832,11 @@
         </is>
       </c>
       <c r="D38" s="11" t="n">
-        <v>28</v>
+        <v>19.5</v>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>48.8%</t>
         </is>
       </c>
       <c r="F38" s="13" t="inlineStr"/>
@@ -1912,11 +1904,11 @@
         </is>
       </c>
       <c r="D40" s="11" t="n">
-        <v>20.5</v>
+        <v>15</v>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>51.2%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="F40" s="13" t="inlineStr"/>
@@ -1984,11 +1976,11 @@
         </is>
       </c>
       <c r="D42" s="11" t="n">
-        <v>36</v>
+        <v>32.5</v>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>90.0%</t>
+          <t>81.2%</t>
         </is>
       </c>
       <c r="F42" s="13" t="inlineStr"/>
@@ -2020,11 +2012,11 @@
         </is>
       </c>
       <c r="D43" s="11" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>77.5%</t>
+          <t>52.5%</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr"/>
@@ -2056,11 +2048,11 @@
         </is>
       </c>
       <c r="D44" s="11" t="n">
-        <v>34.5</v>
+        <v>33.5</v>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>86.2%</t>
+          <t>83.8%</t>
         </is>
       </c>
       <c r="F44" s="13" t="inlineStr"/>
@@ -2092,11 +2084,11 @@
         </is>
       </c>
       <c r="D45" s="11" t="n">
-        <v>37.5</v>
+        <v>38</v>
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>93.8%</t>
+          <t>95.0%</t>
         </is>
       </c>
       <c r="F45" s="13" t="inlineStr"/>
@@ -2164,11 +2156,11 @@
         </is>
       </c>
       <c r="D47" s="11" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E47" s="12" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>82.5%</t>
         </is>
       </c>
       <c r="F47" s="13" t="inlineStr"/>
@@ -2236,11 +2228,11 @@
         </is>
       </c>
       <c r="D49" s="11" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>67.5%</t>
         </is>
       </c>
       <c r="F49" s="13" t="inlineStr"/>
@@ -2272,11 +2264,11 @@
         </is>
       </c>
       <c r="D50" s="11" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>47.5%</t>
         </is>
       </c>
       <c r="F50" s="13" t="inlineStr"/>
@@ -2308,11 +2300,11 @@
         </is>
       </c>
       <c r="D51" s="11" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>47.5%</t>
         </is>
       </c>
       <c r="F51" s="13" t="inlineStr"/>

</xml_diff>

<commit_message>
Match AI benchmark marks with Final Music List listening scores and rank order
</commit_message>
<xml_diff>
--- a/Judges_Scoring_Sheet.xlsx
+++ b/Judges_Scoring_Sheet.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Judges Scoring Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finalists Scoring Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,7 +52,12 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="10"/>
+      <b val="1"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -65,6 +70,10 @@
       <b val="1"/>
       <color rgb="001E3A8A"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="10">
@@ -100,8 +109,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAFAFA"/>
-        <bgColor rgb="00FAFAFA"/>
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -147,23 +156,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00CBD5E1"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00CBD5E1"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00CBD5E1"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00CBD5E1"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -184,37 +193,43 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -585,10 +600,10 @@
   <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
@@ -602,14 +617,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI MUSIC COMPETITION — OFFICIAL JUDGES EVALUATION SHEET (TOTAL: 100 MARKS)</t>
+          <t>AI MUSIC COMPETITION — FINAL MUSIC LIST &amp; JUDGES SCORING SHEET</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Framework: AI Benchmark (40 Marks, Audio-Calibrated) + Human Judges Live Defense (60 Marks: Creativity 20M, Music Composition 20M, Emotional Impact 10M, Presentation 10M)</t>
+          <t>Final Music List (Ranked 1 to 36) | Framework: AI Listening Benchmark (40 Marks) + Human Judges Live Defense (60 Marks) = 100 Marks</t>
         </is>
       </c>
     </row>
@@ -648,12 +663,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Rank</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Team Name</t>
+          <t>Team Name (S.No)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -663,13 +678,13 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>PART A: AI Benchmark (40M)</t>
+          <t>PART A: Listening Benchmark</t>
         </is>
       </c>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>PART B: Human Judges Live Scoring (60M)</t>
+          <t>PART B: Live Human Judges Scoring (60M)</t>
         </is>
       </c>
       <c r="G6" s="6" t="n"/>
@@ -689,8 +704,7 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Judges Defense Remarks &amp; Notes
-(Questions / Strengths / Vulnerabilities)</t>
+          <t>Judges Defense Remarks &amp; Notes</t>
         </is>
       </c>
     </row>
@@ -700,13 +714,12 @@
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>AI Mark
-(/40)</t>
+          <t>Score (/40)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>AI %</t>
+          <t>Rank %</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -738,12 +751,14 @@
       <c r="L7" s="4" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="8" t="n">
-        <v>1</v>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>ajay guptha</t>
+          <t>VisionX (#38)</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -752,11 +767,11 @@
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr"/>
@@ -771,28 +786,30 @@
         <f>IF(J8&lt;&gt;"", D8+J8, D8)</f>
         <v/>
       </c>
-      <c r="L8" s="10" t="inlineStr"/>
+      <c r="L8" s="16" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>Sound Waves</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Mikrokosmos (#41)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D9" s="11" t="n">
-        <v>30.5</v>
+        <v>36.8</v>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>76.2%</t>
+          <t>92.0%</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr"/>
@@ -807,28 +824,30 @@
         <f>IF(J9&lt;&gt;"", D9+J9, D9)</f>
         <v/>
       </c>
-      <c r="L9" s="18" t="inlineStr"/>
+      <c r="L9" s="20" t="inlineStr"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="8" t="n">
-        <v>3</v>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Code &amp; Chords</t>
+          <t>ajay guptha (#01)</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>32.5</v>
+        <v>35.2</v>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>81.2%</t>
+          <t>88.0%</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr"/>
@@ -843,28 +862,30 @@
         <f>IF(J10&lt;&gt;"", D10+J10, D10)</f>
         <v/>
       </c>
-      <c r="L10" s="10" t="inlineStr"/>
+      <c r="L10" s="16" t="inlineStr"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>SYNERA</t>
-        </is>
-      </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>THE SOUNDERS (#40)</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D11" s="11" t="n">
-        <v>28</v>
+        <v>33.6</v>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>84.0%</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr"/>
@@ -879,28 +900,30 @@
         <f>IF(J11&lt;&gt;"", D11+J11, D11)</f>
         <v/>
       </c>
-      <c r="L11" s="18" t="inlineStr"/>
+      <c r="L11" s="20" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="8" t="n">
-        <v>5</v>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>CODE &amp; CHORDS</t>
+          <t>AI MELODY (#25)</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D12" s="11" t="n">
-        <v>31.5</v>
+        <v>32</v>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>78.8%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr"/>
@@ -915,28 +938,34 @@
         <f>IF(J12&lt;&gt;"", D12+J12, D12)</f>
         <v/>
       </c>
-      <c r="L12" s="10" t="inlineStr"/>
+      <c r="L12" s="16" t="inlineStr">
+        <is>
+          <t>song is good,but theme is different</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Code &amp; Chords</t>
-        </is>
-      </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>#6</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Muse Ai (#32)</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
         <is>
           <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D13" s="11" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr"/>
@@ -951,28 +980,30 @@
         <f>IF(J13&lt;&gt;"", D13+J13, D13)</f>
         <v/>
       </c>
-      <c r="L13" s="18" t="inlineStr"/>
+      <c r="L13" s="20" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="8" t="n">
-        <v>7</v>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>#7</t>
+        </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>404TALENTNOTFOUND</t>
+          <t>THE DIGITAL MAESTROS (#39)</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr"/>
@@ -987,28 +1018,30 @@
         <f>IF(J14&lt;&gt;"", D14+J14, D14)</f>
         <v/>
       </c>
-      <c r="L14" s="10" t="inlineStr"/>
+      <c r="L14" s="16" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>Algorythm</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>#8</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>NEUROBEATS (#09)</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
       <c r="D15" s="11" t="n">
-        <v>32.5</v>
+        <v>30.4</v>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>81.2%</t>
+          <t>76.0%</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr"/>
@@ -1023,15 +1056,17 @@
         <f>IF(J15&lt;&gt;"", D15+J15, D15)</f>
         <v/>
       </c>
-      <c r="L15" s="18" t="inlineStr"/>
+      <c r="L15" s="20" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="8" t="n">
-        <v>9</v>
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>#9</t>
+        </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>NEUROBEATS</t>
+          <t>RAAGA (#19)</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -1040,11 +1075,11 @@
         </is>
       </c>
       <c r="D16" s="11" t="n">
-        <v>34.5</v>
+        <v>30.4</v>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>86.2%</t>
+          <t>76.0%</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr"/>
@@ -1059,28 +1094,30 @@
         <f>IF(J16&lt;&gt;"", D16+J16, D16)</f>
         <v/>
       </c>
-      <c r="L16" s="10" t="inlineStr"/>
+      <c r="L16" s="16" t="inlineStr"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>404 Not Found</t>
-        </is>
-      </c>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>Heroes Among us</t>
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>#10</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Trinetras (#37)</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D17" s="11" t="n">
-        <v>23.5</v>
+        <v>30.4</v>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>58.8%</t>
+          <t>76.0%</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr"/>
@@ -1095,28 +1132,30 @@
         <f>IF(J17&lt;&gt;"", D17+J17, D17)</f>
         <v/>
       </c>
-      <c r="L17" s="18" t="inlineStr"/>
+      <c r="L17" s="20" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="8" t="n">
-        <v>11</v>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>#11</t>
+        </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>TEAM JIGS</t>
+          <t>Melody Lemon (#30)</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>26.5</v>
+        <v>29.6</v>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>66.2%</t>
+          <t>74.0%</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr"/>
@@ -1131,28 +1170,30 @@
         <f>IF(J18&lt;&gt;"", D18+J18, D18)</f>
         <v/>
       </c>
-      <c r="L18" s="10" t="inlineStr"/>
+      <c r="L18" s="16" t="inlineStr"/>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="16" t="n">
-        <v>12</v>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>MUSIC QUEENS</t>
-        </is>
-      </c>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>Heroes Among us</t>
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>#12</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Code &amp; Chords (#03)</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D19" s="11" t="n">
-        <v>29</v>
+        <v>28.8</v>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>72.5%</t>
+          <t>72.0%</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr"/>
@@ -1167,28 +1208,30 @@
         <f>IF(J19&lt;&gt;"", D19+J19, D19)</f>
         <v/>
       </c>
-      <c r="L19" s="18" t="inlineStr"/>
+      <c r="L19" s="20" t="inlineStr"/>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="8" t="n">
-        <v>13</v>
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>#12</t>
+        </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>SOLO</t>
+          <t>CODE &amp; CHORDS (#05)</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>25.5</v>
+        <v>28.8</v>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>63.7%</t>
+          <t>72.0%</t>
         </is>
       </c>
       <c r="F20" s="13" t="inlineStr"/>
@@ -1203,28 +1246,30 @@
         <f>IF(J20&lt;&gt;"", D20+J20, D20)</f>
         <v/>
       </c>
-      <c r="L20" s="10" t="inlineStr"/>
+      <c r="L20" s="16" t="inlineStr"/>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="16" t="n">
-        <v>14</v>
-      </c>
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>Single knight</t>
-        </is>
-      </c>
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>Engineering</t>
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>#12</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Code &amp; Chords (#06)</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D21" s="11" t="n">
-        <v>25</v>
+        <v>28.8</v>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>72.0%</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr"/>
@@ -1239,15 +1284,17 @@
         <f>IF(J21&lt;&gt;"", D21+J21, D21)</f>
         <v/>
       </c>
-      <c r="L21" s="18" t="inlineStr"/>
+      <c r="L21" s="20" t="inlineStr"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="8" t="n">
-        <v>15</v>
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>#13</t>
+        </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Kanyarasi</t>
+          <t>TEAM EYES (#17)</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -1256,11 +1303,11 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>24.5</v>
+        <v>28.8</v>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>61.3%</t>
+          <t>72.0%</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr"/>
@@ -1275,28 +1322,30 @@
         <f>IF(J22&lt;&gt;"", D22+J22, D22)</f>
         <v/>
       </c>
-      <c r="L22" s="10" t="inlineStr"/>
+      <c r="L22" s="16" t="inlineStr"/>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>Sonic Innovators</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>Heroes Among us</t>
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>#14</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Sound Waves (#02)</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D23" s="11" t="n">
-        <v>25.5</v>
+        <v>28</v>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>63.7%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr"/>
@@ -1311,28 +1360,30 @@
         <f>IF(J23&lt;&gt;"", D23+J23, D23)</f>
         <v/>
       </c>
-      <c r="L23" s="18" t="inlineStr"/>
+      <c r="L23" s="20" t="inlineStr"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="8" t="n">
-        <v>17</v>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>#17</t>
+        </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>TEAM EYES</t>
+          <t>Algorythm (#08)</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D24" s="11" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>82.5%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="F24" s="13" t="inlineStr"/>
@@ -1347,28 +1398,30 @@
         <f>IF(J24&lt;&gt;"", D24+J24, D24)</f>
         <v/>
       </c>
-      <c r="L24" s="10" t="inlineStr"/>
+      <c r="L24" s="16" t="inlineStr"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="16" t="n">
-        <v>18</v>
-      </c>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>Musical Chairs</t>
-        </is>
-      </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>Heroes Among us</t>
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>#18</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Code slayers (#23)</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="inlineStr">
+        <is>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D25" s="11" t="n">
-        <v>29.5</v>
+        <v>27.2</v>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>73.8%</t>
+          <t>68.0%</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr"/>
@@ -1383,28 +1436,30 @@
         <f>IF(J25&lt;&gt;"", D25+J25, D25)</f>
         <v/>
       </c>
-      <c r="L25" s="18" t="inlineStr"/>
+      <c r="L25" s="20" t="inlineStr"/>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="8" t="n">
-        <v>19</v>
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>#19</t>
+        </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>RAAGA</t>
+          <t>LONGCLAW (#20)</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D26" s="11" t="n">
-        <v>33</v>
+        <v>26.4</v>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>82.5%</t>
+          <t>66.0%</t>
         </is>
       </c>
       <c r="F26" s="13" t="inlineStr"/>
@@ -1419,28 +1474,30 @@
         <f>IF(J26&lt;&gt;"", D26+J26, D26)</f>
         <v/>
       </c>
-      <c r="L26" s="10" t="inlineStr"/>
+      <c r="L26" s="16" t="inlineStr"/>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>LONGCLAW</t>
-        </is>
-      </c>
-      <c r="C27" s="18" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>#20</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>CYBER KNIGHTS (#35)</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D27" s="11" t="n">
-        <v>31</v>
+        <v>25.6</v>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>77.5%</t>
+          <t>64.0%</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr"/>
@@ -1455,28 +1512,30 @@
         <f>IF(J27&lt;&gt;"", D27+J27, D27)</f>
         <v/>
       </c>
-      <c r="L27" s="18" t="inlineStr"/>
+      <c r="L27" s="20" t="inlineStr"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="8" t="n">
-        <v>21</v>
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>#21</t>
+        </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Quantum Minds</t>
+          <t>Cadence (#24)</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>27</v>
+        <v>24.8</v>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>67.5%</t>
+          <t>62.0%</t>
         </is>
       </c>
       <c r="F28" s="13" t="inlineStr"/>
@@ -1491,28 +1550,30 @@
         <f>IF(J28&lt;&gt;"", D28+J28, D28)</f>
         <v/>
       </c>
-      <c r="L28" s="10" t="inlineStr"/>
+      <c r="L28" s="16" t="inlineStr"/>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="16" t="n">
-        <v>22</v>
-      </c>
-      <c r="B29" s="17" t="inlineStr">
-        <is>
-          <t>GUITAR AI</t>
-        </is>
-      </c>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>Engineering</t>
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>#22</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>SYNERA (#04)</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>47.5%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr"/>
@@ -1527,28 +1588,30 @@
         <f>IF(J29&lt;&gt;"", D29+J29, D29)</f>
         <v/>
       </c>
-      <c r="L29" s="18" t="inlineStr"/>
+      <c r="L29" s="20" t="inlineStr"/>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="8" t="n">
-        <v>23</v>
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>#23</t>
+        </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Code slayers</t>
+          <t>Musical Chairs (#18)</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D30" s="11" t="n">
-        <v>30.5</v>
+        <v>24</v>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>76.2%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="F30" s="13" t="inlineStr"/>
@@ -1563,28 +1626,30 @@
         <f>IF(J30&lt;&gt;"", D30+J30, D30)</f>
         <v/>
       </c>
-      <c r="L30" s="10" t="inlineStr"/>
+      <c r="L30" s="16" t="inlineStr"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="16" t="n">
-        <v>24</v>
-      </c>
-      <c r="B31" s="17" t="inlineStr">
-        <is>
-          <t>Cadence</t>
-        </is>
-      </c>
-      <c r="C31" s="18" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>#24</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>MUSIC QUEENS (#12)</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="inlineStr">
+        <is>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D31" s="11" t="n">
-        <v>29.5</v>
+        <v>23.2</v>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>73.8%</t>
+          <t>58.0%</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr"/>
@@ -1599,28 +1664,30 @@
         <f>IF(J31&lt;&gt;"", D31+J31, D31)</f>
         <v/>
       </c>
-      <c r="L31" s="18" t="inlineStr"/>
+      <c r="L31" s="20" t="inlineStr"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="8" t="n">
-        <v>25</v>
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>#25</t>
+        </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>AI MELODY</t>
+          <t>Quantum Minds (#21)</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Heroes Among us</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D32" s="11" t="n">
-        <v>35</v>
+        <v>22.4</v>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>56.0%</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr"/>
@@ -1635,28 +1702,30 @@
         <f>IF(J32&lt;&gt;"", D32+J32, D32)</f>
         <v/>
       </c>
-      <c r="L32" s="10" t="inlineStr"/>
+      <c r="L32" s="16" t="inlineStr"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="16" t="n">
-        <v>26</v>
-      </c>
-      <c r="B33" s="17" t="inlineStr">
-        <is>
-          <t>Melody Minds</t>
-        </is>
-      </c>
-      <c r="C33" s="18" t="inlineStr">
-        <is>
-          <t>Engineering</t>
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>#26</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t>404 Not Found (#10)</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="inlineStr">
+        <is>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D33" s="11" t="n">
-        <v>16</v>
+        <v>20.8</v>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>52.0%</t>
         </is>
       </c>
       <c r="F33" s="13" t="inlineStr"/>
@@ -1671,15 +1740,17 @@
         <f>IF(J33&lt;&gt;"", D33+J33, D33)</f>
         <v/>
       </c>
-      <c r="L33" s="18" t="inlineStr"/>
+      <c r="L33" s="20" t="inlineStr"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="8" t="n">
-        <v>27</v>
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>#27</t>
+        </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Epic beats</t>
+          <t>Utimatrix (#34)</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -1688,11 +1759,11 @@
         </is>
       </c>
       <c r="D34" s="11" t="n">
-        <v>21.5</v>
+        <v>20.8</v>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>53.8%</t>
+          <t>52.0%</t>
         </is>
       </c>
       <c r="F34" s="13" t="inlineStr"/>
@@ -1707,28 +1778,30 @@
         <f>IF(J34&lt;&gt;"", D34+J34, D34)</f>
         <v/>
       </c>
-      <c r="L34" s="10" t="inlineStr"/>
+      <c r="L34" s="16" t="inlineStr"/>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="16" t="n">
-        <v>28</v>
-      </c>
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>AInovators</t>
-        </is>
-      </c>
-      <c r="C35" s="18" t="inlineStr">
-        <is>
-          <t>Heroes Among us</t>
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="B35" s="18" t="inlineStr">
+        <is>
+          <t>404TALENTNOTFOUND (#07)</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D35" s="11" t="n">
-        <v>25.5</v>
+        <v>20</v>
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>63.7%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr"/>
@@ -1743,28 +1816,30 @@
         <f>IF(J35&lt;&gt;"", D35+J35, D35)</f>
         <v/>
       </c>
-      <c r="L35" s="18" t="inlineStr"/>
+      <c r="L35" s="20" t="inlineStr"/>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="8" t="n">
-        <v>29</v>
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>#29</t>
+        </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Melody makers</t>
+          <t>TEAM JIGS (#11)</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Heroes Among us</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D36" s="11" t="n">
-        <v>26</v>
+        <v>19.2</v>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>65.0%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F36" s="13" t="inlineStr"/>
@@ -1779,28 +1854,30 @@
         <f>IF(J36&lt;&gt;"", D36+J36, D36)</f>
         <v/>
       </c>
-      <c r="L36" s="10" t="inlineStr"/>
+      <c r="L36" s="16" t="inlineStr"/>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="16" t="n">
-        <v>30</v>
-      </c>
-      <c r="B37" s="17" t="inlineStr">
-        <is>
-          <t>Melody Lemon</t>
-        </is>
-      </c>
-      <c r="C37" s="18" t="inlineStr">
-        <is>
-          <t>Heroes Among us</t>
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>#30</t>
+        </is>
+      </c>
+      <c r="B37" s="18" t="inlineStr">
+        <is>
+          <t>SOLO (#13)</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr">
+        <is>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D37" s="11" t="n">
-        <v>34.5</v>
+        <v>19.2</v>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>86.2%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F37" s="13" t="inlineStr"/>
@@ -1815,15 +1892,17 @@
         <f>IF(J37&lt;&gt;"", D37+J37, D37)</f>
         <v/>
       </c>
-      <c r="L37" s="18" t="inlineStr"/>
+      <c r="L37" s="20" t="inlineStr"/>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="8" t="n">
-        <v>31</v>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>#31</t>
+        </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>The Boyzz</t>
+          <t>Single knight (#14)</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
@@ -1832,11 +1911,11 @@
         </is>
       </c>
       <c r="D38" s="11" t="n">
-        <v>19.5</v>
+        <v>17.6</v>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>48.8%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="F38" s="13" t="inlineStr"/>
@@ -1851,28 +1930,30 @@
         <f>IF(J38&lt;&gt;"", D38+J38, D38)</f>
         <v/>
       </c>
-      <c r="L38" s="10" t="inlineStr"/>
+      <c r="L38" s="16" t="inlineStr"/>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="16" t="n">
-        <v>32</v>
-      </c>
-      <c r="B39" s="17" t="inlineStr">
-        <is>
-          <t>Muse Ai</t>
-        </is>
-      </c>
-      <c r="C39" s="18" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>#32</t>
+        </is>
+      </c>
+      <c r="B39" s="18" t="inlineStr">
+        <is>
+          <t>Kanyarasi (#15)</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="inlineStr">
         <is>
           <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D39" s="11" t="n">
-        <v>36.5</v>
+        <v>17.6</v>
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>91.2%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="F39" s="13" t="inlineStr"/>
@@ -1887,28 +1968,30 @@
         <f>IF(J39&lt;&gt;"", D39+J39, D39)</f>
         <v/>
       </c>
-      <c r="L39" s="18" t="inlineStr"/>
+      <c r="L39" s="20" t="inlineStr"/>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="8" t="n">
-        <v>33</v>
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>#33</t>
+        </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Musical stars</t>
+          <t>Sonic Innovators (#16)</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D40" s="11" t="n">
-        <v>15</v>
+        <v>16.8</v>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>37.5%</t>
+          <t>42.0%</t>
         </is>
       </c>
       <c r="F40" s="13" t="inlineStr"/>
@@ -1923,28 +2006,30 @@
         <f>IF(J40&lt;&gt;"", D40+J40, D40)</f>
         <v/>
       </c>
-      <c r="L40" s="10" t="inlineStr"/>
+      <c r="L40" s="16" t="inlineStr"/>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="16" t="n">
-        <v>34</v>
-      </c>
-      <c r="B41" s="17" t="inlineStr">
-        <is>
-          <t>Utimatrix</t>
-        </is>
-      </c>
-      <c r="C41" s="18" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>#34</t>
+        </is>
+      </c>
+      <c r="B41" s="18" t="inlineStr">
+        <is>
+          <t>Epic beats (#27)</t>
+        </is>
+      </c>
+      <c r="C41" s="19" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
       <c r="D41" s="11" t="n">
-        <v>37.5</v>
+        <v>16</v>
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>93.8%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F41" s="13" t="inlineStr"/>
@@ -1959,28 +2044,30 @@
         <f>IF(J41&lt;&gt;"", D41+J41, D41)</f>
         <v/>
       </c>
-      <c r="L41" s="18" t="inlineStr"/>
+      <c r="L41" s="20" t="inlineStr"/>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="8" t="n">
-        <v>35</v>
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>#35</t>
+        </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>CYBER KNIGHTS</t>
+          <t>AInovators (#28)</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D42" s="11" t="n">
-        <v>32.5</v>
+        <v>16</v>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>81.2%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F42" s="13" t="inlineStr"/>
@@ -1995,28 +2082,30 @@
         <f>IF(J42&lt;&gt;"", D42+J42, D42)</f>
         <v/>
       </c>
-      <c r="L42" s="10" t="inlineStr"/>
+      <c r="L42" s="16" t="inlineStr"/>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="16" t="n">
-        <v>36</v>
-      </c>
-      <c r="B43" s="17" t="inlineStr">
-        <is>
-          <t>SoulSync</t>
-        </is>
-      </c>
-      <c r="C43" s="18" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t>Melody makers (#29)</t>
+        </is>
+      </c>
+      <c r="C43" s="19" t="inlineStr">
+        <is>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D43" s="11" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>52.5%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr"/>
@@ -2031,28 +2120,30 @@
         <f>IF(J43&lt;&gt;"", D43+J43, D43)</f>
         <v/>
       </c>
-      <c r="L43" s="18" t="inlineStr"/>
+      <c r="L43" s="20" t="inlineStr"/>
     </row>
     <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="8" t="n">
-        <v>37</v>
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Trinetras</t>
+          <t>GUITAR AI (#22)</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D44" s="11" t="n">
-        <v>33.5</v>
+        <v>12</v>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>83.8%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="F44" s="13" t="inlineStr"/>
@@ -2067,28 +2158,34 @@
         <f>IF(J44&lt;&gt;"", D44+J44, D44)</f>
         <v/>
       </c>
-      <c r="L44" s="10" t="inlineStr"/>
+      <c r="L44" s="16" t="inlineStr">
+        <is>
+          <t>Not shortlisted in Final Music List due to flat audio execution.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="16" t="n">
-        <v>38</v>
-      </c>
-      <c r="B45" s="17" t="inlineStr">
-        <is>
-          <t>VisionX</t>
-        </is>
-      </c>
-      <c r="C45" s="18" t="inlineStr">
-        <is>
-          <t>Heroes Among us</t>
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="inlineStr">
+        <is>
+          <t>Melody Minds (#26)</t>
+        </is>
+      </c>
+      <c r="C45" s="19" t="inlineStr">
+        <is>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D45" s="11" t="n">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>95.0%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="F45" s="13" t="inlineStr"/>
@@ -2103,28 +2200,34 @@
         <f>IF(J45&lt;&gt;"", D45+J45, D45)</f>
         <v/>
       </c>
-      <c r="L45" s="18" t="inlineStr"/>
+      <c r="L45" s="20" t="inlineStr">
+        <is>
+          <t>Not shortlisted in Final Music List due to flat audio execution.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="8" t="n">
-        <v>39</v>
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>THE DIGITAL MAESTROS</t>
+          <t>The Boyzz (#31)</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>Heroes Among us</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D46" s="11" t="n">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>85.0%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="F46" s="13" t="inlineStr"/>
@@ -2139,28 +2242,34 @@
         <f>IF(J46&lt;&gt;"", D46+J46, D46)</f>
         <v/>
       </c>
-      <c r="L46" s="10" t="inlineStr"/>
+      <c r="L46" s="16" t="inlineStr">
+        <is>
+          <t>Not shortlisted in Final Music List due to flat audio execution.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="16" t="n">
-        <v>40</v>
-      </c>
-      <c r="B47" s="17" t="inlineStr">
-        <is>
-          <t>THE SOUNDERS</t>
-        </is>
-      </c>
-      <c r="C47" s="18" t="inlineStr">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>Musical stars (#33)</t>
+        </is>
+      </c>
+      <c r="C47" s="19" t="inlineStr">
         <is>
           <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D47" s="11" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="E47" s="12" t="inlineStr">
         <is>
-          <t>82.5%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="F47" s="13" t="inlineStr"/>
@@ -2175,15 +2284,21 @@
         <f>IF(J47&lt;&gt;"", D47+J47, D47)</f>
         <v/>
       </c>
-      <c r="L47" s="18" t="inlineStr"/>
+      <c r="L47" s="20" t="inlineStr">
+        <is>
+          <t>Not shortlisted in Final Music List due to flat audio execution.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="8" t="n">
-        <v>41</v>
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Mikrokosmos</t>
+          <t>SoulSync (#36)</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
@@ -2192,11 +2307,11 @@
         </is>
       </c>
       <c r="D48" s="11" t="n">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>92.5%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="F48" s="13" t="inlineStr"/>
@@ -2211,28 +2326,34 @@
         <f>IF(J48&lt;&gt;"", D48+J48, D48)</f>
         <v/>
       </c>
-      <c r="L48" s="10" t="inlineStr"/>
+      <c r="L48" s="16" t="inlineStr">
+        <is>
+          <t>Not shortlisted in Final Music List due to flat audio execution.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="16" t="n">
-        <v>42</v>
-      </c>
-      <c r="B49" s="17" t="inlineStr">
-        <is>
-          <t>Think Twice</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>Think Twice (#42)</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
       <c r="D49" s="11" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>67.5%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F49" s="13" t="inlineStr"/>
@@ -2247,15 +2368,21 @@
         <f>IF(J49&lt;&gt;"", D49+J49, D49)</f>
         <v/>
       </c>
-      <c r="L49" s="18" t="inlineStr"/>
+      <c r="L49" s="20" t="inlineStr">
+        <is>
+          <t>Evaluated as Irrelevant to announced theme during listening.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="8" t="n">
-        <v>43</v>
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>Coders</t>
+          <t>Coders (#43)</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
@@ -2264,11 +2391,11 @@
         </is>
       </c>
       <c r="D50" s="11" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>47.5%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="F50" s="13" t="inlineStr"/>
@@ -2283,28 +2410,34 @@
         <f>IF(J50&lt;&gt;"", D50+J50, D50)</f>
         <v/>
       </c>
-      <c r="L50" s="10" t="inlineStr"/>
+      <c r="L50" s="16" t="inlineStr">
+        <is>
+          <t>Evaluated as Irrelevant to theme during audio listening.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="16" t="n">
-        <v>44</v>
-      </c>
-      <c r="B51" s="17" t="inlineStr">
-        <is>
-          <t>Byteforce</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>Byteforce (#44)</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
       <c r="D51" s="11" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>47.5%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="F51" s="13" t="inlineStr"/>
@@ -2319,7 +2452,11 @@
         <f>IF(J51&lt;&gt;"", D51+J51, D51)</f>
         <v/>
       </c>
-      <c r="L51" s="18" t="inlineStr"/>
+      <c r="L51" s="20" t="inlineStr">
+        <is>
+          <t>Fail (10/50): College fest DJ party track with zero engineering problem-solving.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">

</xml_diff>

<commit_message>
Deploy 36 Finalists Live Stage and Eliminated Teams Archive page
</commit_message>
<xml_diff>
--- a/Judges_Scoring_Sheet.xlsx
+++ b/Judges_Scoring_Sheet.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finalists Scoring Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="36 Finalists Scoring Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -597,11 +597,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
@@ -617,14 +617,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI MUSIC COMPETITION — FINAL MUSIC LIST &amp; JUDGES SCORING SHEET</t>
+          <t>AI MUSIC COMPETITION — 36 FINALISTS OFFICIAL JUDGES SCORING SHEET</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Final Music List (Ranked 1 to 36) | Framework: AI Listening Benchmark (40 Marks) + Human Judges Live Defense (60 Marks) = 100 Marks</t>
+          <t>36 Finalists | Framework: AI Benchmark (40 Marks) + Human Judges Live Defense (60 Marks: Creativity 20M, Composition 20M, Emotion 10M, Presentation 10M) = 100 Marks</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Team Name (S.No)</t>
+          <t>Team Name (Orig. S.No)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>PART A: Listening Benchmark</t>
+          <t>PART A: AI Benchmark (40M)</t>
         </is>
       </c>
       <c r="E6" s="5" t="n"/>
@@ -753,7 +753,7 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>#1</t>
+          <t>#01</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -791,7 +791,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>#2</t>
+          <t>#02</t>
         </is>
       </c>
       <c r="B9" s="18" t="inlineStr">
@@ -829,7 +829,7 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>#3</t>
+          <t>#03</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -867,7 +867,7 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>#4</t>
+          <t>#04</t>
         </is>
       </c>
       <c r="B11" s="18" t="inlineStr">
@@ -905,7 +905,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>#5</t>
+          <t>#05</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>#6</t>
+          <t>#06</t>
         </is>
       </c>
       <c r="B13" s="18" t="inlineStr">
@@ -985,7 +985,7 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>#7</t>
+          <t>#07</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -1023,7 +1023,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>#8</t>
+          <t>#08</t>
         </is>
       </c>
       <c r="B15" s="18" t="inlineStr">
@@ -1061,7 +1061,7 @@
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>#9</t>
+          <t>#09</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -1213,12 +1213,12 @@
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>#12</t>
+          <t>#13</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>CODE &amp; CHORDS (#05)</t>
+          <t>TEAM EYES (#17)</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -1251,12 +1251,12 @@
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>#12</t>
+          <t>#14</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>Code &amp; Chords (#06)</t>
+          <t>Sound Waves (#02)</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
@@ -1265,11 +1265,11 @@
         </is>
       </c>
       <c r="D21" s="11" t="n">
-        <v>28.8</v>
+        <v>28</v>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>72.0%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr"/>
@@ -1289,12 +1289,12 @@
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>#13</t>
+          <t>#15</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>TEAM EYES (#17)</t>
+          <t>CODE &amp; CHORDS (#05)</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -1303,11 +1303,11 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>28.8</v>
+        <v>28</v>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>72.0%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr"/>
@@ -1327,12 +1327,12 @@
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>#14</t>
+          <t>#16</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>Sound Waves (#02)</t>
+          <t>Code &amp; Chords (#06)</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
@@ -2121,342 +2121,6 @@
         <v/>
       </c>
       <c r="L43" s="20" t="inlineStr"/>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B44" s="9" t="inlineStr">
-        <is>
-          <t>GUITAR AI (#22)</t>
-        </is>
-      </c>
-      <c r="C44" s="10" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="D44" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="E44" s="12" t="inlineStr">
-        <is>
-          <t>30.0%</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="inlineStr"/>
-      <c r="G44" s="13" t="inlineStr"/>
-      <c r="H44" s="13" t="inlineStr"/>
-      <c r="I44" s="13" t="inlineStr"/>
-      <c r="J44" s="14">
-        <f>IF(COUNT(F44:I44)&gt;0, SUM(F44:I44), "")</f>
-        <v/>
-      </c>
-      <c r="K44" s="15">
-        <f>IF(J44&lt;&gt;"", D44+J44, D44)</f>
-        <v/>
-      </c>
-      <c r="L44" s="16" t="inlineStr">
-        <is>
-          <t>Not shortlisted in Final Music List due to flat audio execution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B45" s="18" t="inlineStr">
-        <is>
-          <t>Melody Minds (#26)</t>
-        </is>
-      </c>
-      <c r="C45" s="19" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="D45" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="E45" s="12" t="inlineStr">
-        <is>
-          <t>30.0%</t>
-        </is>
-      </c>
-      <c r="F45" s="13" t="inlineStr"/>
-      <c r="G45" s="13" t="inlineStr"/>
-      <c r="H45" s="13" t="inlineStr"/>
-      <c r="I45" s="13" t="inlineStr"/>
-      <c r="J45" s="14">
-        <f>IF(COUNT(F45:I45)&gt;0, SUM(F45:I45), "")</f>
-        <v/>
-      </c>
-      <c r="K45" s="15">
-        <f>IF(J45&lt;&gt;"", D45+J45, D45)</f>
-        <v/>
-      </c>
-      <c r="L45" s="20" t="inlineStr">
-        <is>
-          <t>Not shortlisted in Final Music List due to flat audio execution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>The Boyzz (#31)</t>
-        </is>
-      </c>
-      <c r="C46" s="10" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="D46" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="E46" s="12" t="inlineStr">
-        <is>
-          <t>30.0%</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="inlineStr"/>
-      <c r="G46" s="13" t="inlineStr"/>
-      <c r="H46" s="13" t="inlineStr"/>
-      <c r="I46" s="13" t="inlineStr"/>
-      <c r="J46" s="14">
-        <f>IF(COUNT(F46:I46)&gt;0, SUM(F46:I46), "")</f>
-        <v/>
-      </c>
-      <c r="K46" s="15">
-        <f>IF(J46&lt;&gt;"", D46+J46, D46)</f>
-        <v/>
-      </c>
-      <c r="L46" s="16" t="inlineStr">
-        <is>
-          <t>Not shortlisted in Final Music List due to flat audio execution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B47" s="18" t="inlineStr">
-        <is>
-          <t>Musical stars (#33)</t>
-        </is>
-      </c>
-      <c r="C47" s="19" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
-        </is>
-      </c>
-      <c r="D47" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t>30.0%</t>
-        </is>
-      </c>
-      <c r="F47" s="13" t="inlineStr"/>
-      <c r="G47" s="13" t="inlineStr"/>
-      <c r="H47" s="13" t="inlineStr"/>
-      <c r="I47" s="13" t="inlineStr"/>
-      <c r="J47" s="14">
-        <f>IF(COUNT(F47:I47)&gt;0, SUM(F47:I47), "")</f>
-        <v/>
-      </c>
-      <c r="K47" s="15">
-        <f>IF(J47&lt;&gt;"", D47+J47, D47)</f>
-        <v/>
-      </c>
-      <c r="L47" s="20" t="inlineStr">
-        <is>
-          <t>Not shortlisted in Final Music List due to flat audio execution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>SoulSync (#36)</t>
-        </is>
-      </c>
-      <c r="C48" s="10" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>30.0%</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="inlineStr"/>
-      <c r="G48" s="13" t="inlineStr"/>
-      <c r="H48" s="13" t="inlineStr"/>
-      <c r="I48" s="13" t="inlineStr"/>
-      <c r="J48" s="14">
-        <f>IF(COUNT(F48:I48)&gt;0, SUM(F48:I48), "")</f>
-        <v/>
-      </c>
-      <c r="K48" s="15">
-        <f>IF(J48&lt;&gt;"", D48+J48, D48)</f>
-        <v/>
-      </c>
-      <c r="L48" s="16" t="inlineStr">
-        <is>
-          <t>Not shortlisted in Final Music List due to flat audio execution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B49" s="18" t="inlineStr">
-        <is>
-          <t>Think Twice (#42)</t>
-        </is>
-      </c>
-      <c r="C49" s="19" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="E49" s="12" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="F49" s="13" t="inlineStr"/>
-      <c r="G49" s="13" t="inlineStr"/>
-      <c r="H49" s="13" t="inlineStr"/>
-      <c r="I49" s="13" t="inlineStr"/>
-      <c r="J49" s="14">
-        <f>IF(COUNT(F49:I49)&gt;0, SUM(F49:I49), "")</f>
-        <v/>
-      </c>
-      <c r="K49" s="15">
-        <f>IF(J49&lt;&gt;"", D49+J49, D49)</f>
-        <v/>
-      </c>
-      <c r="L49" s="20" t="inlineStr">
-        <is>
-          <t>Evaluated as Irrelevant to announced theme during listening.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>Coders (#43)</t>
-        </is>
-      </c>
-      <c r="C50" s="10" t="inlineStr">
-        <is>
-          <t>Heroes Among us</t>
-        </is>
-      </c>
-      <c r="D50" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="E50" s="12" t="inlineStr">
-        <is>
-          <t>30.0%</t>
-        </is>
-      </c>
-      <c r="F50" s="13" t="inlineStr"/>
-      <c r="G50" s="13" t="inlineStr"/>
-      <c r="H50" s="13" t="inlineStr"/>
-      <c r="I50" s="13" t="inlineStr"/>
-      <c r="J50" s="14">
-        <f>IF(COUNT(F50:I50)&gt;0, SUM(F50:I50), "")</f>
-        <v/>
-      </c>
-      <c r="K50" s="15">
-        <f>IF(J50&lt;&gt;"", D50+J50, D50)</f>
-        <v/>
-      </c>
-      <c r="L50" s="16" t="inlineStr">
-        <is>
-          <t>Evaluated as Irrelevant to theme during audio listening.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B51" s="18" t="inlineStr">
-        <is>
-          <t>Byteforce (#44)</t>
-        </is>
-      </c>
-      <c r="C51" s="19" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="D51" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="E51" s="12" t="inlineStr">
-        <is>
-          <t>20.0%</t>
-        </is>
-      </c>
-      <c r="F51" s="13" t="inlineStr"/>
-      <c r="G51" s="13" t="inlineStr"/>
-      <c r="H51" s="13" t="inlineStr"/>
-      <c r="I51" s="13" t="inlineStr"/>
-      <c r="J51" s="14">
-        <f>IF(COUNT(F51:I51)&gt;0, SUM(F51:I51), "")</f>
-        <v/>
-      </c>
-      <c r="K51" s="15">
-        <f>IF(J51&lt;&gt;"", D51+J51, D51)</f>
-        <v/>
-      </c>
-      <c r="L51" s="20" t="inlineStr">
-        <is>
-          <t>Fail (10/50): College fest DJ party track with zero engineering problem-solving.</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="13">

</xml_diff>

<commit_message>
Update Judges Scoring Sheet sorted by Team Number with Team # column
</commit_message>
<xml_diff>
--- a/Judges_Scoring_Sheet.xlsx
+++ b/Judges_Scoring_Sheet.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="36 Finalists Scoring Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Judges Scoring Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +53,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="9.5"/>
     </font>
     <font>
@@ -76,7 +82,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +111,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="0092400E"/>
         <bgColor rgb="0092400E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -172,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -196,40 +208,37 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -600,7 +609,7 @@
   <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -617,14 +626,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI MUSIC COMPETITION — 36 FINALISTS OFFICIAL JUDGES SCORING SHEET</t>
+          <t>AI MUSIC COMPETITION — OFFICIAL JUDGES SCORING SHEET (SORTED BY TEAM NUMBER)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>36 Finalists | Framework: AI Benchmark (40 Marks) + Human Judges Live Defense (60 Marks: Creativity 20M, Composition 20M, Emotion 10M, Presentation 10M) = 100 Marks</t>
+          <t>36 Finalists (Sorted #01 to #41) | Framework: AI Benchmark (40 Marks) + Human Judges Live Defense (60 Marks: Creativity 20M, Composition 20M, Emotion 10M, Presentation 10M) = 100 Marks</t>
         </is>
       </c>
     </row>
@@ -663,12 +672,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Rank</t>
+          <t>Team #</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Team Name (Orig. S.No)</t>
+          <t>Team Name</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -719,7 +728,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Rank %</t>
+          <t>AI %</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -758,7 +767,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>VisionX (#38)</t>
+          <t>ajay guptha</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -767,11 +776,11 @@
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>40</v>
+        <v>35.2</v>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>88.0%</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr"/>
@@ -789,27 +798,27 @@
       <c r="L8" s="16" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>#02</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Mikrokosmos (#41)</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Sound Waves</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D9" s="11" t="n">
-        <v>36.8</v>
+        <v>28</v>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>92.0%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr"/>
@@ -824,7 +833,7 @@
         <f>IF(J9&lt;&gt;"", D9+J9, D9)</f>
         <v/>
       </c>
-      <c r="L9" s="20" t="inlineStr"/>
+      <c r="L9" s="19" t="inlineStr"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -834,20 +843,20 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>ajay guptha (#01)</t>
+          <t>Code &amp; Chords</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Heroes Among us</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>35.2</v>
+        <v>28.8</v>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>88.0%</t>
+          <t>72.0%</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr"/>
@@ -865,27 +874,27 @@
       <c r="L10" s="16" t="inlineStr"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>#04</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>THE SOUNDERS (#40)</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>SYNERA</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D11" s="11" t="n">
-        <v>33.6</v>
+        <v>24</v>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>84.0%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr"/>
@@ -900,7 +909,7 @@
         <f>IF(J11&lt;&gt;"", D11+J11, D11)</f>
         <v/>
       </c>
-      <c r="L11" s="20" t="inlineStr"/>
+      <c r="L11" s="19" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -910,20 +919,20 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>AI MELODY (#25)</t>
+          <t>CODE &amp; CHORDS</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Heroes Among us</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D12" s="11" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr"/>
@@ -938,34 +947,30 @@
         <f>IF(J12&lt;&gt;"", D12+J12, D12)</f>
         <v/>
       </c>
-      <c r="L12" s="16" t="inlineStr">
-        <is>
-          <t>song is good,but theme is different</t>
-        </is>
-      </c>
+      <c r="L12" s="16" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>#06</t>
         </is>
       </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Muse Ai (#32)</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Code &amp; Chords</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D13" s="11" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr"/>
@@ -980,7 +985,7 @@
         <f>IF(J13&lt;&gt;"", D13+J13, D13)</f>
         <v/>
       </c>
-      <c r="L13" s="20" t="inlineStr"/>
+      <c r="L13" s="19" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -990,20 +995,20 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>THE DIGITAL MAESTROS (#39)</t>
+          <t>404TALENTNOTFOUND</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>Heroes Among us</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr"/>
@@ -1021,27 +1026,27 @@
       <c r="L14" s="16" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>#08</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>NEUROBEATS (#09)</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Algorythm</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
       <c r="D15" s="11" t="n">
-        <v>30.4</v>
+        <v>28</v>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>76.0%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr"/>
@@ -1056,7 +1061,7 @@
         <f>IF(J15&lt;&gt;"", D15+J15, D15)</f>
         <v/>
       </c>
-      <c r="L15" s="20" t="inlineStr"/>
+      <c r="L15" s="19" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -1066,7 +1071,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>RAAGA (#19)</t>
+          <t>NEUROBEATS</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -1097,27 +1102,27 @@
       <c r="L16" s="16" t="inlineStr"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>#10</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Trinetras (#37)</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>404 Not Found</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D17" s="11" t="n">
-        <v>30.4</v>
+        <v>20.8</v>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>76.0%</t>
+          <t>52.0%</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr"/>
@@ -1132,7 +1137,7 @@
         <f>IF(J17&lt;&gt;"", D17+J17, D17)</f>
         <v/>
       </c>
-      <c r="L17" s="20" t="inlineStr"/>
+      <c r="L17" s="19" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -1142,20 +1147,20 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Melody Lemon (#30)</t>
+          <t>TEAM JIGS</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Heroes Among us</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>29.6</v>
+        <v>19.2</v>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>74.0%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr"/>
@@ -1173,27 +1178,27 @@
       <c r="L18" s="16" t="inlineStr"/>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>#12</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>Code &amp; Chords (#03)</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>MUSIC QUEENS</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D19" s="11" t="n">
-        <v>28.8</v>
+        <v>23.2</v>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>72.0%</t>
+          <t>58.0%</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr"/>
@@ -1208,7 +1213,7 @@
         <f>IF(J19&lt;&gt;"", D19+J19, D19)</f>
         <v/>
       </c>
-      <c r="L19" s="20" t="inlineStr"/>
+      <c r="L19" s="19" t="inlineStr"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -1218,20 +1223,20 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>TEAM EYES (#17)</t>
+          <t>SOLO</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>28.8</v>
+        <v>19.2</v>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>72.0%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F20" s="13" t="inlineStr"/>
@@ -1249,27 +1254,27 @@
       <c r="L20" s="16" t="inlineStr"/>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>#14</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>Sound Waves (#02)</t>
-        </is>
-      </c>
-      <c r="C21" s="19" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Single knight</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D21" s="11" t="n">
-        <v>28</v>
+        <v>17.6</v>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr"/>
@@ -1284,7 +1289,7 @@
         <f>IF(J21&lt;&gt;"", D21+J21, D21)</f>
         <v/>
       </c>
-      <c r="L21" s="20" t="inlineStr"/>
+      <c r="L21" s="19" t="inlineStr"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -1294,7 +1299,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>CODE &amp; CHORDS (#05)</t>
+          <t>Kanyarasi</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -1303,11 +1308,11 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>28</v>
+        <v>17.6</v>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr"/>
@@ -1325,27 +1330,27 @@
       <c r="L22" s="16" t="inlineStr"/>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>#16</t>
         </is>
       </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Code &amp; Chords (#06)</t>
-        </is>
-      </c>
-      <c r="C23" s="19" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>Sonic Innovators</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D23" s="11" t="n">
-        <v>28</v>
+        <v>16.8</v>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>42.0%</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr"/>
@@ -1360,7 +1365,7 @@
         <f>IF(J23&lt;&gt;"", D23+J23, D23)</f>
         <v/>
       </c>
-      <c r="L23" s="20" t="inlineStr"/>
+      <c r="L23" s="19" t="inlineStr"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -1370,20 +1375,20 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Algorythm (#08)</t>
+          <t>TEAM EYES</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D24" s="11" t="n">
-        <v>28</v>
+        <v>28.8</v>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>72.0%</t>
         </is>
       </c>
       <c r="F24" s="13" t="inlineStr"/>
@@ -1401,27 +1406,27 @@
       <c r="L24" s="16" t="inlineStr"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>#18</t>
         </is>
       </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Code slayers (#23)</t>
-        </is>
-      </c>
-      <c r="C25" s="19" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Musical Chairs</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D25" s="11" t="n">
-        <v>27.2</v>
+        <v>24</v>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>68.0%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr"/>
@@ -1436,7 +1441,7 @@
         <f>IF(J25&lt;&gt;"", D25+J25, D25)</f>
         <v/>
       </c>
-      <c r="L25" s="20" t="inlineStr"/>
+      <c r="L25" s="19" t="inlineStr"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -1446,20 +1451,20 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>LONGCLAW (#20)</t>
+          <t>RAAGA</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D26" s="11" t="n">
-        <v>26.4</v>
+        <v>30.4</v>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>66.0%</t>
+          <t>76.0%</t>
         </is>
       </c>
       <c r="F26" s="13" t="inlineStr"/>
@@ -1477,27 +1482,27 @@
       <c r="L26" s="16" t="inlineStr"/>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="17" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>#20</t>
         </is>
       </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>CYBER KNIGHTS (#35)</t>
-        </is>
-      </c>
-      <c r="C27" s="19" t="inlineStr">
-        <is>
-          <t>Engineering</t>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>LONGCLAW</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D27" s="11" t="n">
-        <v>25.6</v>
+        <v>26.4</v>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>64.0%</t>
+          <t>66.0%</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr"/>
@@ -1512,7 +1517,7 @@
         <f>IF(J27&lt;&gt;"", D27+J27, D27)</f>
         <v/>
       </c>
-      <c r="L27" s="20" t="inlineStr"/>
+      <c r="L27" s="19" t="inlineStr"/>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -1522,20 +1527,20 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Cadence (#24)</t>
+          <t>Quantum Minds</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>The Greatest Gift</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>24.8</v>
+        <v>22.4</v>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>62.0%</t>
+          <t>56.0%</t>
         </is>
       </c>
       <c r="F28" s="13" t="inlineStr"/>
@@ -1553,27 +1558,27 @@
       <c r="L28" s="16" t="inlineStr"/>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="17" t="inlineStr">
-        <is>
-          <t>#22</t>
-        </is>
-      </c>
-      <c r="B29" s="18" t="inlineStr">
-        <is>
-          <t>SYNERA (#04)</t>
-        </is>
-      </c>
-      <c r="C29" s="19" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>#23</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Code slayers</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>24</v>
+        <v>27.2</v>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>68.0%</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr"/>
@@ -1588,30 +1593,30 @@
         <f>IF(J29&lt;&gt;"", D29+J29, D29)</f>
         <v/>
       </c>
-      <c r="L29" s="20" t="inlineStr"/>
+      <c r="L29" s="19" t="inlineStr"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>#23</t>
+          <t>#24</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Musical Chairs (#18)</t>
+          <t>Cadence</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Heroes Among us</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D30" s="11" t="n">
-        <v>24</v>
+        <v>24.8</v>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>62.0%</t>
         </is>
       </c>
       <c r="F30" s="13" t="inlineStr"/>
@@ -1629,27 +1634,27 @@
       <c r="L30" s="16" t="inlineStr"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="17" t="inlineStr">
-        <is>
-          <t>#24</t>
-        </is>
-      </c>
-      <c r="B31" s="18" t="inlineStr">
-        <is>
-          <t>MUSIC QUEENS (#12)</t>
-        </is>
-      </c>
-      <c r="C31" s="19" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>#25</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>AI MELODY</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D31" s="11" t="n">
-        <v>23.2</v>
+        <v>32</v>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr"/>
@@ -1664,17 +1669,21 @@
         <f>IF(J31&lt;&gt;"", D31+J31, D31)</f>
         <v/>
       </c>
-      <c r="L31" s="20" t="inlineStr"/>
+      <c r="L31" s="19" t="inlineStr">
+        <is>
+          <t>song is good,but theme is different</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>#25</t>
+          <t>#27</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Quantum Minds (#21)</t>
+          <t>Epic beats</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
@@ -1683,11 +1692,11 @@
         </is>
       </c>
       <c r="D32" s="11" t="n">
-        <v>22.4</v>
+        <v>16</v>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>56.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr"/>
@@ -1705,27 +1714,27 @@
       <c r="L32" s="16" t="inlineStr"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="17" t="inlineStr">
-        <is>
-          <t>#26</t>
-        </is>
-      </c>
-      <c r="B33" s="18" t="inlineStr">
-        <is>
-          <t>404 Not Found (#10)</t>
-        </is>
-      </c>
-      <c r="C33" s="19" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>AInovators</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D33" s="11" t="n">
-        <v>20.8</v>
+        <v>16</v>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F33" s="13" t="inlineStr"/>
@@ -1740,30 +1749,30 @@
         <f>IF(J33&lt;&gt;"", D33+J33, D33)</f>
         <v/>
       </c>
-      <c r="L33" s="20" t="inlineStr"/>
+      <c r="L33" s="19" t="inlineStr"/>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>#27</t>
+          <t>#29</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Utimatrix (#34)</t>
+          <t>Melody makers</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D34" s="11" t="n">
-        <v>20.8</v>
+        <v>16</v>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F34" s="13" t="inlineStr"/>
@@ -1781,27 +1790,27 @@
       <c r="L34" s="16" t="inlineStr"/>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="17" t="inlineStr">
-        <is>
-          <t>#28</t>
-        </is>
-      </c>
-      <c r="B35" s="18" t="inlineStr">
-        <is>
-          <t>404TALENTNOTFOUND (#07)</t>
-        </is>
-      </c>
-      <c r="C35" s="19" t="inlineStr">
-        <is>
-          <t>The Greatest Gift</t>
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>#30</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Melody Lemon</t>
+        </is>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D35" s="11" t="n">
-        <v>20</v>
+        <v>29.6</v>
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>74.0%</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr"/>
@@ -1816,17 +1825,17 @@
         <f>IF(J35&lt;&gt;"", D35+J35, D35)</f>
         <v/>
       </c>
-      <c r="L35" s="20" t="inlineStr"/>
+      <c r="L35" s="19" t="inlineStr"/>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>#29</t>
+          <t>#32</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>TEAM JIGS (#11)</t>
+          <t>Muse Ai</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
@@ -1835,11 +1844,11 @@
         </is>
       </c>
       <c r="D36" s="11" t="n">
-        <v>19.2</v>
+        <v>32</v>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="F36" s="13" t="inlineStr"/>
@@ -1857,27 +1866,27 @@
       <c r="L36" s="16" t="inlineStr"/>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="17" t="inlineStr">
-        <is>
-          <t>#30</t>
-        </is>
-      </c>
-      <c r="B37" s="18" t="inlineStr">
-        <is>
-          <t>SOLO (#13)</t>
-        </is>
-      </c>
-      <c r="C37" s="19" t="inlineStr">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>#34</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>Utimatrix</t>
+        </is>
+      </c>
+      <c r="C37" s="18" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
       <c r="D37" s="11" t="n">
-        <v>19.2</v>
+        <v>20.8</v>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>52.0%</t>
         </is>
       </c>
       <c r="F37" s="13" t="inlineStr"/>
@@ -1892,17 +1901,17 @@
         <f>IF(J37&lt;&gt;"", D37+J37, D37)</f>
         <v/>
       </c>
-      <c r="L37" s="20" t="inlineStr"/>
+      <c r="L37" s="19" t="inlineStr"/>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>#31</t>
+          <t>#35</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Single knight (#14)</t>
+          <t>CYBER KNIGHTS</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
@@ -1911,11 +1920,11 @@
         </is>
       </c>
       <c r="D38" s="11" t="n">
-        <v>17.6</v>
+        <v>25.6</v>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>44.0%</t>
+          <t>64.0%</t>
         </is>
       </c>
       <c r="F38" s="13" t="inlineStr"/>
@@ -1933,27 +1942,27 @@
       <c r="L38" s="16" t="inlineStr"/>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="17" t="inlineStr">
-        <is>
-          <t>#32</t>
-        </is>
-      </c>
-      <c r="B39" s="18" t="inlineStr">
-        <is>
-          <t>Kanyarasi (#15)</t>
-        </is>
-      </c>
-      <c r="C39" s="19" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>#37</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>Trinetras</t>
+        </is>
+      </c>
+      <c r="C39" s="18" t="inlineStr">
         <is>
           <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D39" s="11" t="n">
-        <v>17.6</v>
+        <v>30.4</v>
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>44.0%</t>
+          <t>76.0%</t>
         </is>
       </c>
       <c r="F39" s="13" t="inlineStr"/>
@@ -1968,17 +1977,17 @@
         <f>IF(J39&lt;&gt;"", D39+J39, D39)</f>
         <v/>
       </c>
-      <c r="L39" s="20" t="inlineStr"/>
+      <c r="L39" s="19" t="inlineStr"/>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>#33</t>
+          <t>#38</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Sonic Innovators (#16)</t>
+          <t>VisionX</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
@@ -1987,11 +1996,11 @@
         </is>
       </c>
       <c r="D40" s="11" t="n">
-        <v>16.8</v>
+        <v>40</v>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>42.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="F40" s="13" t="inlineStr"/>
@@ -2009,27 +2018,27 @@
       <c r="L40" s="16" t="inlineStr"/>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="17" t="inlineStr">
-        <is>
-          <t>#34</t>
-        </is>
-      </c>
-      <c r="B41" s="18" t="inlineStr">
-        <is>
-          <t>Epic beats (#27)</t>
-        </is>
-      </c>
-      <c r="C41" s="19" t="inlineStr">
-        <is>
-          <t>Engineering</t>
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>#39</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>THE DIGITAL MAESTROS</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>Heroes Among us</t>
         </is>
       </c>
       <c r="D41" s="11" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="F41" s="13" t="inlineStr"/>
@@ -2044,30 +2053,30 @@
         <f>IF(J41&lt;&gt;"", D41+J41, D41)</f>
         <v/>
       </c>
-      <c r="L41" s="20" t="inlineStr"/>
+      <c r="L41" s="19" t="inlineStr"/>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>#35</t>
+          <t>#40</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>AInovators (#28)</t>
+          <t>THE SOUNDERS</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>Heroes Among us</t>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D42" s="11" t="n">
-        <v>16</v>
+        <v>33.6</v>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>84.0%</t>
         </is>
       </c>
       <c r="F42" s="13" t="inlineStr"/>
@@ -2085,27 +2094,27 @@
       <c r="L42" s="16" t="inlineStr"/>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="17" t="inlineStr">
-        <is>
-          <t>#36</t>
-        </is>
-      </c>
-      <c r="B43" s="18" t="inlineStr">
-        <is>
-          <t>Melody makers (#29)</t>
-        </is>
-      </c>
-      <c r="C43" s="19" t="inlineStr">
-        <is>
-          <t>Heroes Among us</t>
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>#41</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>Mikrokosmos</t>
+        </is>
+      </c>
+      <c r="C43" s="18" t="inlineStr">
+        <is>
+          <t>The Greatest Gift</t>
         </is>
       </c>
       <c r="D43" s="11" t="n">
-        <v>16</v>
+        <v>36.8</v>
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>92.0%</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr"/>
@@ -2120,7 +2129,7 @@
         <f>IF(J43&lt;&gt;"", D43+J43, D43)</f>
         <v/>
       </c>
-      <c r="L43" s="20" t="inlineStr"/>
+      <c r="L43" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="13">

</xml_diff>